<commit_message>
feat: update actual spend to use demo excel expense tracker and clean sheets
</commit_message>
<xml_diff>
--- a/frontend/public/sample-docs/73 Broadway.xlsx
+++ b/frontend/public/sample-docs/73 Broadway.xlsx
@@ -3,17 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Partnership ration &amp; funding" sheetId="1" r:id="rId1"/>
-    <sheet name="Inner Bank Transfer" sheetId="2" r:id="rId2"/>
-    <sheet name="Columbia Bank" sheetId="3" r:id="rId3"/>
-    <sheet name="Total Expenses" sheetId="4" r:id="rId4"/>
-    <sheet name="Construction Exp" sheetId="5" r:id="rId5"/>
-    <sheet name="Labour Exp" sheetId="6" r:id="rId6"/>
-    <sheet name="Accounting &amp; Legal exp" sheetId="7" r:id="rId7"/>
-    <sheet name="Bank Fee" sheetId="8" r:id="rId8"/>
-    <sheet name="Muncipality Exp" sheetId="9" r:id="rId9"/>
-    <sheet name="Misc Exp" sheetId="10" r:id="rId10"/>
-    <sheet name="Land Acquisition" sheetId="11" r:id="rId11"/>
+    <sheet name="Total Expenses" sheetId="1" r:id="rId1"/>
+    <sheet name="Construction Exp" sheetId="2" r:id="rId2"/>
+    <sheet name="Labour Exp" sheetId="3" r:id="rId3"/>
+    <sheet name="Accounting &amp; Legal fee" sheetId="4" r:id="rId4"/>
+    <sheet name="Bank Fee" sheetId="5" r:id="rId5"/>
+    <sheet name="Municipal Exp" sheetId="6" r:id="rId6"/>
+    <sheet name="Misc Exp" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -407,249 +403,248 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Partner Name</v>
+        <v>SR. NO</v>
       </c>
       <c r="B1" t="str">
-        <v>Allocation Ratio</v>
+        <v>Type</v>
       </c>
       <c r="C1" t="str">
-        <v>Capital Commitment</v>
+        <v>Amount</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>Marcus Vance</v>
-      </c>
-      <c r="B2">
-        <v>0.25</v>
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Construction Exp</v>
       </c>
       <c r="C2">
-        <v>200000</v>
+        <v>656154.06</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>Elena Rostova</v>
-      </c>
-      <c r="B3">
-        <v>0.25</v>
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Labour Exp</v>
       </c>
       <c r="C3">
-        <v>200000</v>
+        <v>73406.5</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>Apex Equity Capital</v>
-      </c>
-      <c r="B4">
-        <v>0.25</v>
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Accounting &amp; Legal fee</v>
       </c>
       <c r="C4">
-        <v>200000</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>Horizon Development Partners LLC</v>
-      </c>
-      <c r="B5">
-        <v>0.25</v>
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Bank Fee</v>
       </c>
       <c r="C5">
-        <v>200000</v>
+        <v>581.51</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Municipal Exp</v>
+      </c>
+      <c r="C6">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Misc Exp</v>
+      </c>
+      <c r="C7">
+        <v>334649.93</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Date</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Mode</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Description</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Amount</v>
-      </c>
-      <c r="E1" t="str">
-        <v/>
-      </c>
-      <c r="F1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="G1">
-        <v>-150735.16</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>46059</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Credit</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Contingency Return Deposit</v>
-      </c>
-      <c r="D2">
-        <v>-150735.16</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Date</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Mode</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Description</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Amount</v>
-      </c>
-      <c r="E1" t="str">
-        <v/>
-      </c>
-      <c r="F1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="G1">
-        <v>725399.82</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>45730</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Debit</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Commercial Land Acquisition Deposit</v>
-      </c>
-      <c r="D2">
-        <v>90000</v>
-      </c>
-      <c r="E2" t="str">
-        <v>DEPOSIT</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>45751</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Debit</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Commercial Escrow Closing Wire</v>
-      </c>
-      <c r="D3">
-        <v>635399.82</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:G10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Date</v>
       </c>
       <c r="B1" t="str">
-        <v>Amount Total</v>
+        <v>Mode</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v>Total</v>
+      </c>
+      <c r="G1">
+        <v>656154.06</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v/>
+      <c r="A2">
+        <v>45845</v>
       </c>
       <c r="B2" t="str">
-        <v>Operating Account</v>
+        <v>PO-301</v>
       </c>
       <c r="C2" t="str">
-        <v>Escrow Reserve</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Capital Sweeps</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Capex Reserve</v>
+        <v>Apex Structural Steel Supply &amp; Erect</v>
+      </c>
+      <c r="D2">
+        <v>185000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>45791</v>
-      </c>
-      <c r="B3">
-        <v>50000</v>
-      </c>
-      <c r="C3">
-        <v>-50000</v>
+        <v>45859</v>
+      </c>
+      <c r="B3" t="str">
+        <v>PO-302</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Carrier Mechanical &amp; HVAC Equipment</v>
       </c>
       <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>45798</v>
-      </c>
-      <c r="B4">
-        <v>-50000</v>
-      </c>
-      <c r="C4">
-        <v>50000</v>
+        <v>45890</v>
+      </c>
+      <c r="B4" t="str">
+        <v>PO-303</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Artisan Architectural Woodwork &amp; Millwork</v>
       </c>
       <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>45910</v>
+      </c>
+      <c r="B5" t="str">
+        <v>PO-304</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Peak Engineering &amp; Structural Testing</v>
+      </c>
+      <c r="D5">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>45930</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Inv #HV-2025-01</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Horizon HVAC Rough Installation</v>
+      </c>
+      <c r="D6">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>45960</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Inv #HV-2025-02</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Horizon Electrical Conduit &amp; Panels</v>
+      </c>
+      <c r="D7">
+        <v>65000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>45990</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Inv #AC-441</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Apex Framing Supply &amp; Lumbers</v>
+      </c>
+      <c r="D8">
+        <v>78000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>46010</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Inv #104</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Broadway Framing Package Labor Phase 1</v>
+      </c>
+      <c r="D9">
+        <v>54000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>46030</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Inv #109</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Broadway Framing Package Labor Phase 2</v>
+      </c>
+      <c r="D10">
+        <v>54154.06</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -678,49 +673,49 @@
         <v>Total</v>
       </c>
       <c r="G1">
-        <v>-400000</v>
+        <v>73406.5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>43957</v>
+        <v>45846</v>
       </c>
       <c r="B2" t="str">
-        <v>Credit</v>
+        <v>Check 1275</v>
       </c>
       <c r="C2" t="str">
-        <v>Lender Construction Advance #1</v>
+        <v>Certified Framing Trade Crew</v>
       </c>
       <c r="D2">
-        <v>-100000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>46199</v>
+        <v>45950</v>
       </c>
       <c r="B3" t="str">
-        <v>Credit</v>
+        <v>Check 1041</v>
       </c>
       <c r="C3" t="str">
-        <v>Lender Construction Advance #2</v>
+        <v>Mechanical Subcontractor Labor</v>
       </c>
       <c r="D3">
-        <v>-200000</v>
+        <v>28406.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>46254</v>
+        <v>46062</v>
       </c>
       <c r="B4" t="str">
-        <v>Credit</v>
+        <v>Check 1054</v>
       </c>
       <c r="C4" t="str">
-        <v>Lender Construction Advance #3</v>
+        <v>Electrical Rough-in Crew</v>
       </c>
       <c r="D4">
-        <v>-100000</v>
+        <v>20000</v>
       </c>
     </row>
   </sheetData>
@@ -732,95 +727,69 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>SR. NO</v>
+        <v>Date</v>
       </c>
       <c r="B1" t="str">
-        <v>Type</v>
+        <v>Mode</v>
       </c>
       <c r="C1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="D1" t="str">
         <v>Amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v>Total</v>
+      </c>
+      <c r="G1">
+        <v>1750</v>
       </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>1</v>
+        <v>46092</v>
       </c>
       <c r="B2" t="str">
-        <v>Construction Cost</v>
-      </c>
-      <c r="C2">
-        <v>656154.06</v>
+        <v>Debit</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Institutional Construction Audit CPA</v>
+      </c>
+      <c r="D2">
+        <v>750</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>2</v>
+        <v>46204</v>
       </c>
       <c r="B3" t="str">
-        <v>Bank fees</v>
-      </c>
-      <c r="C3">
-        <v>581.51</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Muncipality</v>
-      </c>
-      <c r="C4">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Subcontractor Labor</v>
-      </c>
-      <c r="C5">
-        <v>73406.5</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Accounting &amp; Legal</v>
-      </c>
-      <c r="C6">
-        <v>1750</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Land Acquisition</v>
-      </c>
-      <c r="C7">
-        <v>725399.82</v>
+        <v>Debit</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Project Legal &amp; Title Review Counsel</v>
+      </c>
+      <c r="D3">
+        <v>1000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -842,138 +811,54 @@
         <v>Total</v>
       </c>
       <c r="G1">
-        <v>656154.06</v>
+        <v>581.51</v>
       </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>45845</v>
+        <v>45751</v>
       </c>
       <c r="B2" t="str">
-        <v>PO-301</v>
+        <v>Debit</v>
       </c>
       <c r="C2" t="str">
-        <v>Apex Structural Steel Supply &amp; Erect</v>
+        <v>Commercial Wire Transfer Fee</v>
       </c>
       <c r="D2">
-        <v>185000</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>45859</v>
+        <v>45768</v>
       </c>
       <c r="B3" t="str">
-        <v>PO-302</v>
+        <v>Debit</v>
       </c>
       <c r="C3" t="str">
-        <v>Carrier Mechanical &amp; HVAC Equipment</v>
+        <v>Commercial Wire Transfer Fee</v>
       </c>
       <c r="D3">
-        <v>95000</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>45890</v>
+        <v>45770</v>
       </c>
       <c r="B4" t="str">
-        <v>PO-303</v>
+        <v>Debit</v>
       </c>
       <c r="C4" t="str">
-        <v>Artisan Architectural Woodwork &amp; Millwork</v>
+        <v>Escrow Disbursement Maintenance Fee</v>
       </c>
       <c r="D4">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>45910</v>
-      </c>
-      <c r="B5" t="str">
-        <v>PO-304</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Peak Engineering &amp; Structural Testing</v>
-      </c>
-      <c r="D5">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>45930</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Inv #HV-2025-01</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Horizon HVAC Rough Installation</v>
-      </c>
-      <c r="D6">
-        <v>55000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>45960</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Inv #HV-2025-02</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Horizon Electrical Conduit &amp; Panels</v>
-      </c>
-      <c r="D7">
-        <v>65000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>45990</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Inv #AC-441</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Apex Framing Supply &amp; Lumbers</v>
-      </c>
-      <c r="D8">
-        <v>78000</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>46010</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Inv #104</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Broadway Framing Package Labor Phase 1</v>
-      </c>
-      <c r="D9">
-        <v>54000</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>46030</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Inv #109</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Broadway Framing Package Labor Phase 2</v>
-      </c>
-      <c r="D10">
-        <v>54154.06</v>
+        <v>541.51</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1002,49 +887,49 @@
         <v>Total</v>
       </c>
       <c r="G1">
-        <v>73406.5</v>
+        <v>378</v>
       </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>45846</v>
+        <v>45841</v>
       </c>
       <c r="B2" t="str">
-        <v>Check 1275</v>
+        <v>Debit</v>
       </c>
       <c r="C2" t="str">
-        <v>Certified Framing Trade Crew</v>
+        <v>Municipal Department of Buildings Plan Filing</v>
       </c>
       <c r="D2">
-        <v>25000</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>45950</v>
+        <v>46071</v>
       </c>
       <c r="B3" t="str">
-        <v>Check 1041</v>
+        <v>Debit</v>
       </c>
       <c r="C3" t="str">
-        <v>Mechanical Subcontractor Labor</v>
+        <v>Municipal Water &amp; Sewer Inspection</v>
       </c>
       <c r="D3">
-        <v>28406.5</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>46062</v>
+        <v>46077</v>
       </c>
       <c r="B4" t="str">
-        <v>Check 1054</v>
+        <v>Debit</v>
       </c>
       <c r="C4" t="str">
-        <v>Electrical Rough-in Crew</v>
+        <v>Municipal Environmental Sign-off</v>
       </c>
       <c r="D4">
-        <v>20000</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1056,68 +941,6 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Date</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Mode</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Description</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Amount</v>
-      </c>
-      <c r="E1" t="str">
-        <v/>
-      </c>
-      <c r="F1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="G1">
-        <v>1750</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>46092</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Debit</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Institutional Construction Audit CPA</v>
-      </c>
-      <c r="D2">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>46204</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Debit</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Project Legal &amp; Title Review Counsel</v>
-      </c>
-      <c r="D3">
-        <v>1000</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
   <sheetData>
     <row r="1">
@@ -1140,125 +963,49 @@
         <v>Total</v>
       </c>
       <c r="G1">
-        <v>581.51</v>
+        <v>334649.93</v>
       </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>45751</v>
+        <v>45820</v>
       </c>
       <c r="B2" t="str">
-        <v>Debit</v>
+        <v>Check 1001</v>
       </c>
       <c r="C2" t="str">
-        <v>Commercial Wire Transfer Fee</v>
+        <v>Jobsite Facilities, Office Trailer &amp; Security</v>
       </c>
       <c r="D2">
-        <v>20</v>
+        <v>114649.93</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>45768</v>
+        <v>45900</v>
       </c>
       <c r="B3" t="str">
         <v>Debit</v>
       </c>
       <c r="C3" t="str">
-        <v>Commercial Wire Transfer Fee</v>
+        <v>Temporary Site Utilities &amp; Power Hookups</v>
       </c>
       <c r="D3">
-        <v>20</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>45770</v>
+        <v>46000</v>
       </c>
       <c r="B4" t="str">
-        <v>Debit</v>
+        <v>Wire</v>
       </c>
       <c r="C4" t="str">
-        <v>Escrow Disbursement Maintenance Fee</v>
+        <v>Field Superintendent &amp; General Conditions Carry</v>
       </c>
       <c r="D4">
-        <v>541.51</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Date</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Mode</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Description</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Amount</v>
-      </c>
-      <c r="E1" t="str">
-        <v/>
-      </c>
-      <c r="F1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="G1">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>45841</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Debit</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Municipal Department of Buildings Plan Filing</v>
-      </c>
-      <c r="D2">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>46071</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Debit</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Municipal Water &amp; Sewer Inspection</v>
-      </c>
-      <c r="D3">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>46077</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Debit</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Municipal Environmental Sign-off</v>
-      </c>
-      <c r="D4">
-        <v>126</v>
+        <v>100000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>